<commit_message>
Apple-style feel: add apple-design skill and restyle the interface
- Add .claude/skills/apple-design (MIT, from emilkowalski/skills) so future
  interface changes follow it
- Instant press feedback on buttons, chips, rota cells and list rows
- Translucent header; sheets and dialogs materialise when opened and close
  the way they came in
- Phones: edit panel and sign-in become bottom sheets with a grabber; drag
  tracks 1:1, rubber-bands at the top, and a flick (momentum projection)
  closes them, otherwise they spring back
- Size-specific type tracking and leading; system font instead of web fonts
  (no third-party requests, tighter content security policy)
- Gentler fallbacks for reduced motion, reduced transparency and high contrast

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R8EjimpErkij9gvKaTvnbV
</commit_message>
<xml_diff>
--- a/templates/oncall-import-template.xlsx
+++ b/templates/oncall-import-template.xlsx
@@ -127,7 +127,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -142,7 +142,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -157,7 +157,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -172,7 +172,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>46310</v>
+        <v>46317</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -187,7 +187,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <v>46311</v>
+        <v>46318</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -202,7 +202,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -217,7 +217,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>46311</v>
+        <v>46318</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -232,7 +232,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2">
-        <v>46312</v>
+        <v>46319</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -247,7 +247,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2">
-        <v>46313</v>
+        <v>46320</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -262,7 +262,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2">
-        <v>46312</v>
+        <v>46319</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -341,7 +341,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>46307</v>
+        <v>46314</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -356,7 +356,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <v>46308</v>
+        <v>46315</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -376,7 +376,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>46309</v>
+        <v>46316</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -391,7 +391,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>46310</v>
+        <v>46317</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -406,7 +406,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <v>46311</v>
+        <v>46318</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -421,7 +421,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <v>46312</v>
+        <v>46319</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -436,7 +436,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>46313</v>
+        <v>46320</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>

</xml_diff>